<commit_message>
update stopper values, tweaks
</commit_message>
<xml_diff>
--- a/PrincetonReverbUpdate_quantities.xlsx
+++ b/PrincetonReverbUpdate_quantities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Tristan/GitRepos/PrincetonReverbUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{4295EF05-EFBD-FF45-855A-B0E0BBAA6296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{550CA703-50A7-0F41-B404-8C992FBC66D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="1620" windowWidth="27240" windowHeight="15400" xr2:uid="{08900FD0-1E8A-2542-887C-6248B3584EC5}"/>
+    <workbookView xWindow="380" yWindow="620" windowWidth="28040" windowHeight="16400" xr2:uid="{C9D8A07A-9045-7644-9E1A-C7B95F745CC7}"/>
   </bookViews>
   <sheets>
     <sheet name="PrincetonReverbUpdate_quantitie" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
   <si>
     <t>Reference</t>
   </si>
@@ -31,30 +31,30 @@
     <t>Value</t>
   </si>
   <si>
-    <t>R4,R5,R11,R14,R18,R25,R32</t>
+    <t>R3,R6,R21,R23,R24,R31,R45</t>
+  </si>
+  <si>
+    <t>1Meg</t>
+  </si>
+  <si>
+    <t>C1,C2,C7,C9,C12,C24,C29</t>
+  </si>
+  <si>
+    <t>22u 50V</t>
+  </si>
+  <si>
+    <t>R7,R8,R13,R16,R20,R39</t>
+  </si>
+  <si>
+    <t>100k</t>
+  </si>
+  <si>
+    <t>R4,R5,R11,R14,R18</t>
   </si>
   <si>
     <t>1.5k</t>
   </si>
   <si>
-    <t>C1,C2,C7,C9,C12,C24,C29</t>
-  </si>
-  <si>
-    <t>22u 50V</t>
-  </si>
-  <si>
-    <t>R7,R8,R13,R16,R20,R39</t>
-  </si>
-  <si>
-    <t>100k</t>
-  </si>
-  <si>
-    <t>R3,R6,R21,R23,R24,R31</t>
-  </si>
-  <si>
-    <t>1Meg</t>
-  </si>
-  <si>
     <t>C8,C14,C15,C17,C19</t>
   </si>
   <si>
@@ -67,18 +67,24 @@
     <t>220k</t>
   </si>
   <si>
+    <t>R2,R25,R32,R35</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>D1,D3,D4,D5</t>
+  </si>
+  <si>
+    <t>UF4007</t>
+  </si>
+  <si>
     <t>R9,R40,R41</t>
   </si>
   <si>
     <t>10k 3W</t>
   </si>
   <si>
-    <t>D1,D3,D4</t>
-  </si>
-  <si>
-    <t>UF4007</t>
-  </si>
-  <si>
     <t>C18,C23,C25</t>
   </si>
   <si>
@@ -91,12 +97,24 @@
     <t>47n 630V</t>
   </si>
   <si>
+    <t>U5,U6</t>
+  </si>
+  <si>
+    <t>6V6</t>
+  </si>
+  <si>
     <t>RV1,RV5</t>
   </si>
   <si>
     <t>250k Log</t>
   </si>
   <si>
+    <t>R42,R43</t>
+  </si>
+  <si>
+    <t>1k 3W</t>
+  </si>
+  <si>
     <t>R36,R38</t>
   </si>
   <si>
@@ -109,114 +127,108 @@
     <t>56k</t>
   </si>
   <si>
+    <t>C4,C22</t>
+  </si>
+  <si>
+    <t>100n 630V</t>
+  </si>
+  <si>
+    <t>TP2</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>TP1</t>
+  </si>
+  <si>
+    <t>BiasTP</t>
+  </si>
+  <si>
+    <t>RV7</t>
+  </si>
+  <si>
+    <t>22k Lin</t>
+  </si>
+  <si>
+    <t>RV6</t>
+  </si>
+  <si>
+    <t>3M RLog</t>
+  </si>
+  <si>
+    <t>RV4</t>
+  </si>
+  <si>
+    <t>250k Lin</t>
+  </si>
+  <si>
+    <t>RV3</t>
+  </si>
+  <si>
+    <t>100k Log</t>
+  </si>
+  <si>
+    <t>RV2</t>
+  </si>
+  <si>
+    <t>1M Log</t>
+  </si>
+  <si>
+    <t>R48</t>
+  </si>
+  <si>
+    <t>1r 1%</t>
+  </si>
+  <si>
+    <t>R46</t>
+  </si>
+  <si>
+    <t>220k 3W</t>
+  </si>
+  <si>
+    <t>R44</t>
+  </si>
+  <si>
+    <t>680r 5W</t>
+  </si>
+  <si>
+    <t>R37</t>
+  </si>
+  <si>
+    <t>100k 1W</t>
+  </si>
+  <si>
+    <t>R28</t>
+  </si>
+  <si>
+    <t>10k 1W</t>
+  </si>
+  <si>
+    <t>R26</t>
+  </si>
+  <si>
     <t>1k</t>
   </si>
   <si>
-    <t>R17,R45</t>
+    <t>R22</t>
+  </si>
+  <si>
+    <t>2.7k</t>
+  </si>
+  <si>
+    <t>R19</t>
+  </si>
+  <si>
+    <t>47r</t>
+  </si>
+  <si>
+    <t>R17</t>
   </si>
   <si>
     <t>470k</t>
   </si>
   <si>
-    <t>R2,R35</t>
-  </si>
-  <si>
-    <t>10k</t>
-  </si>
-  <si>
-    <t>C4,C22</t>
-  </si>
-  <si>
-    <t>100n 630V</t>
-  </si>
-  <si>
-    <t>TP2</t>
-  </si>
-  <si>
-    <t>GND</t>
-  </si>
-  <si>
-    <t>TP1</t>
-  </si>
-  <si>
-    <t>BiasTP</t>
-  </si>
-  <si>
-    <t>RV7</t>
-  </si>
-  <si>
-    <t>22k Lin</t>
-  </si>
-  <si>
-    <t>RV6</t>
-  </si>
-  <si>
-    <t>3M RLog</t>
-  </si>
-  <si>
-    <t>RV4</t>
-  </si>
-  <si>
-    <t>250k Lin</t>
-  </si>
-  <si>
-    <t>RV3</t>
-  </si>
-  <si>
-    <t>100k Log</t>
-  </si>
-  <si>
-    <t>RV2</t>
-  </si>
-  <si>
-    <t>1M Log</t>
-  </si>
-  <si>
-    <t>R48</t>
-  </si>
-  <si>
-    <t>1r 1%</t>
-  </si>
-  <si>
-    <t>R46</t>
-  </si>
-  <si>
-    <t>220k 3W</t>
-  </si>
-  <si>
-    <t>R44</t>
-  </si>
-  <si>
-    <t>680r 5W</t>
-  </si>
-  <si>
-    <t>1k 3W</t>
-  </si>
-  <si>
-    <t>R37</t>
-  </si>
-  <si>
-    <t>100k 1W</t>
-  </si>
-  <si>
-    <t>R28</t>
-  </si>
-  <si>
-    <t>10k 1W</t>
-  </si>
-  <si>
-    <t>R22</t>
-  </si>
-  <si>
-    <t>2.7k</t>
-  </si>
-  <si>
-    <t>R19</t>
-  </si>
-  <si>
-    <t>47r</t>
-  </si>
-  <si>
     <t>R15</t>
   </si>
   <si>
@@ -244,7 +256,7 @@
     <t>C27</t>
   </si>
   <si>
-    <t>100-470p</t>
+    <t>100p</t>
   </si>
   <si>
     <t>C16</t>
@@ -281,24 +293,6 @@
   </si>
   <si>
     <t>250p 500V</t>
-  </si>
-  <si>
-    <t>Actual in hand</t>
-  </si>
-  <si>
-    <t>2 of the 7 are 6V6 grid stoppers</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>R26</t>
-  </si>
-  <si>
-    <t>R42,R43</t>
-  </si>
-  <si>
-    <t>use 3W?</t>
   </si>
 </sst>
 </file>
@@ -1158,14 +1152,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B584AB2-BCBB-C14D-AD9B-BE3C1B54E736}">
-  <dimension ref="A1:E44"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E25EE3A7-2B38-1644-9FC1-A53A1642091B}">
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1175,14 +1169,8 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1192,14 +1180,8 @@
       <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="D2">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1210,7 +1192,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1220,25 +1202,19 @@
       <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="D4">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="D5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1249,7 +1225,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1259,36 +1235,30 @@
       <c r="C7" t="s">
         <v>14</v>
       </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="s">
         <v>16</v>
       </c>
-      <c r="D8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1299,7 +1269,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1310,18 +1280,18 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>23</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1331,11 +1301,8 @@
       <c r="C13" t="s">
         <v>26</v>
       </c>
-      <c r="D13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1345,383 +1312,349 @@
       <c r="C14" t="s">
         <v>28</v>
       </c>
-      <c r="D14">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
       <c r="C15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16">
         <v>2</v>
       </c>
       <c r="C16" t="s">
-        <v>31</v>
-      </c>
-      <c r="D16">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18">
         <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19">
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B20">
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21">
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B22">
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B24">
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B25">
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
-      </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B27">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
-      </c>
-      <c r="D27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B28">
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>55</v>
-      </c>
-      <c r="D28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>56</v>
-      </c>
-      <c r="D29">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>58</v>
-      </c>
-      <c r="D30">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>60</v>
-      </c>
-      <c r="D31">
-        <v>1</v>
-      </c>
-      <c r="E31" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>62</v>
-      </c>
-      <c r="D32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B33">
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>64</v>
-      </c>
-      <c r="D33">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B34">
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>66</v>
-      </c>
-      <c r="D34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B35">
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
-      </c>
-      <c r="D35">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B36">
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B37">
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B38">
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B39">
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B40">
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B41">
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B43">
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B44">
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>86</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>89</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update bias dropping resistor
</commit_message>
<xml_diff>
--- a/PrincetonReverbUpdate_quantities.xlsx
+++ b/PrincetonReverbUpdate_quantities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Tristan/GitRepos/PrincetonReverbUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{550CA703-50A7-0F41-B404-8C992FBC66D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1516548F-C64D-8F47-AC9A-5EC64F2B0159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="620" windowWidth="28040" windowHeight="16400" xr2:uid="{C9D8A07A-9045-7644-9E1A-C7B95F745CC7}"/>
+    <workbookView xWindow="380" yWindow="620" windowWidth="28040" windowHeight="16400" xr2:uid="{69D57C17-029D-7546-85BE-01358227F806}"/>
   </bookViews>
   <sheets>
     <sheet name="PrincetonReverbUpdate_quantitie" sheetId="1" r:id="rId1"/>
@@ -49,6 +49,12 @@
     <t>100k</t>
   </si>
   <si>
+    <t>R2,R25,R32,R35,R47,R49</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
     <t>R4,R5,R11,R14,R18</t>
   </si>
   <si>
@@ -67,12 +73,6 @@
     <t>220k</t>
   </si>
   <si>
-    <t>R2,R25,R32,R35</t>
-  </si>
-  <si>
-    <t>10k</t>
-  </si>
-  <si>
     <t>D1,D3,D4,D5</t>
   </si>
   <si>
@@ -196,7 +196,7 @@
     <t>R37</t>
   </si>
   <si>
-    <t>100k 1W</t>
+    <t>82k 1W</t>
   </si>
   <si>
     <t>R28</t>
@@ -1152,12 +1152,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E25EE3A7-2B38-1644-9FC1-A53A1642091B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2830297B-7654-2249-BD09-4694B357A20A}">
   <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="24.6640625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1208,7 +1205,7 @@
         <v>9</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
@@ -1230,7 +1227,7 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7" t="s">
         <v>14</v>

</xml_diff>